<commit_message>
rules updates to include WS
</commit_message>
<xml_diff>
--- a/Indmødetal/Regler til Mie.xlsx
+++ b/Indmødetal/Regler til Mie.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://serwizsystems.sharepoint.com/sites/DataogDigitalisering/Delte dokumenter/01_Lufthavn/Indmødetal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="382" documentId="8_{BD8435A5-424E-4FC5-929C-3243556E6BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85ECCD1A-C83F-4C3D-A610-D3BAE0421B4F}"/>
+  <xr:revisionPtr revIDLastSave="389" documentId="8_{BD8435A5-424E-4FC5-929C-3243556E6BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87C19EE6-88D8-4F99-8344-432D29E54C38}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{724EF2EA-7AA9-48FA-9EA3-9140F0F4E3A1}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{724EF2EA-7AA9-48FA-9EA3-9140F0F4E3A1}"/>
   </bookViews>
   <sheets>
     <sheet name="wb" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="71">
   <si>
     <t>Tider WB Clean, search, guard</t>
   </si>
@@ -439,6 +439,9 @@
   <si>
     <t>VL</t>
   </si>
+  <si>
+    <t>WS</t>
+  </si>
 </sst>
 </file>
 
@@ -1046,8 +1049,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{62A5947B-93BF-4B94-A9B6-6F653D116F37}" name="Tabel1" displayName="Tabel1" ref="A1:H69" totalsRowShown="0" headerRowDxfId="9" tableBorderDxfId="8">
-  <autoFilter ref="A1:H69" xr:uid="{62A5947B-93BF-4B94-A9B6-6F653D116F37}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{62A5947B-93BF-4B94-A9B6-6F653D116F37}" name="Tabel1" displayName="Tabel1" ref="A1:H70" totalsRowShown="0" headerRowDxfId="9" tableBorderDxfId="8">
+  <autoFilter ref="A1:H70" xr:uid="{62A5947B-93BF-4B94-A9B6-6F653D116F37}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H37">
     <sortCondition ref="B1:B37"/>
   </sortState>
@@ -1383,13 +1386,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4A27A0D-8896-47A0-95A9-30DD4012C6C3}">
   <dimension ref="B2:J19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="9" max="9" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="54" t="s">
         <v>0</v>
       </c>
@@ -1400,7 +1403,7 @@
       <c r="G2" s="54"/>
       <c r="H2" s="54"/>
     </row>
-    <row r="3" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
@@ -1429,7 +1432,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B4" s="25" t="s">
         <v>9</v>
       </c>
@@ -1454,7 +1457,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="36" t="s">
         <v>9</v>
       </c>
@@ -1481,7 +1484,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="37" t="s">
         <v>9</v>
       </c>
@@ -1504,7 +1507,7 @@
       <c r="I6" s="41"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="25" t="s">
         <v>13</v>
       </c>
@@ -1527,7 +1530,7 @@
       <c r="I7" s="11"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="36" t="s">
         <v>13</v>
       </c>
@@ -1552,7 +1555,7 @@
       </c>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="37" t="s">
         <v>13</v>
       </c>
@@ -1575,7 +1578,7 @@
       <c r="I9" s="41"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="25" t="s">
         <v>15</v>
       </c>
@@ -1598,7 +1601,7 @@
       <c r="I10" s="11"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="36" t="s">
         <v>15</v>
       </c>
@@ -1623,7 +1626,7 @@
       </c>
       <c r="J11" s="1"/>
     </row>
-    <row r="12" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="37" t="s">
         <v>15</v>
       </c>
@@ -1646,7 +1649,7 @@
       <c r="I12" s="42"/>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="29" t="s">
         <v>16</v>
       </c>
@@ -1669,7 +1672,7 @@
       <c r="I13" s="15"/>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="21"/>
       <c r="C14" s="21" t="s">
         <v>18</v>
@@ -1690,7 +1693,7 @@
       <c r="I14" s="16"/>
       <c r="J14" s="1"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="21" t="s">
         <v>19</v>
       </c>
@@ -1713,7 +1716,7 @@
       <c r="I15" s="16"/>
       <c r="J15" s="1"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="21" t="s">
         <v>21</v>
       </c>
@@ -1738,7 +1741,7 @@
       </c>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="2"/>
@@ -1749,7 +1752,7 @@
       <c r="I17" s="12"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C19" s="43" t="s">
         <v>62</v>
       </c>
@@ -1771,13 +1774,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D18F845-7CC0-4A12-B855-0E9D257F383F}">
-  <dimension ref="A1:H69"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H70"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="8" width="12.33203125" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>1</v>
       </c>
@@ -1803,7 +1806,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>35</v>
@@ -1821,7 +1824,7 @@
       </c>
       <c r="H2" s="32"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>47</v>
@@ -1839,7 +1842,7 @@
       </c>
       <c r="H3" s="32"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>39</v>
@@ -1857,7 +1860,7 @@
       </c>
       <c r="H4" s="32"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>41</v>
@@ -1875,7 +1878,7 @@
       </c>
       <c r="H5" s="32"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>59</v>
@@ -1893,7 +1896,7 @@
       </c>
       <c r="H6" s="32"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>33</v>
@@ -1911,7 +1914,7 @@
       </c>
       <c r="H7" s="32"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>58</v>
       </c>
@@ -1931,7 +1934,7 @@
       </c>
       <c r="H8" s="32"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>57</v>
       </c>
@@ -1951,7 +1954,7 @@
       </c>
       <c r="H9" s="32"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>339</v>
       </c>
@@ -1973,7 +1976,7 @@
       </c>
       <c r="H10" s="32"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>333</v>
       </c>
@@ -1995,7 +1998,7 @@
       </c>
       <c r="H11" s="32"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>330</v>
       </c>
@@ -2017,7 +2020,7 @@
       </c>
       <c r="H12" s="32"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
         <v>46</v>
@@ -2035,7 +2038,7 @@
       </c>
       <c r="H13" s="32"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
         <v>55</v>
@@ -2055,7 +2058,7 @@
       </c>
       <c r="H14" s="32"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
         <v>42</v>
@@ -2073,7 +2076,7 @@
       </c>
       <c r="H15" s="32"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
         <v>25</v>
@@ -2091,7 +2094,7 @@
       </c>
       <c r="H16" s="32"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>56</v>
       </c>
@@ -2111,7 +2114,7 @@
       </c>
       <c r="H17" s="32"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
         <v>52</v>
@@ -2129,7 +2132,7 @@
       </c>
       <c r="H18" s="32"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
         <v>48</v>
@@ -2147,7 +2150,7 @@
       </c>
       <c r="H19" s="32"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
         <v>50</v>
@@ -2165,7 +2168,7 @@
       </c>
       <c r="H20" s="32"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
         <v>26</v>
@@ -2183,7 +2186,7 @@
       </c>
       <c r="H21" s="32"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
         <v>49</v>
@@ -2201,7 +2204,7 @@
       </c>
       <c r="H22" s="32"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
         <v>28</v>
@@ -2219,7 +2222,7 @@
       </c>
       <c r="H23" s="32"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
         <v>43</v>
@@ -2237,7 +2240,7 @@
       </c>
       <c r="H24" s="32"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
         <v>29</v>
@@ -2255,7 +2258,7 @@
       </c>
       <c r="H25" s="32"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1" t="s">
         <v>27</v>
@@ -2273,7 +2276,7 @@
       </c>
       <c r="H26" s="32"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
         <v>51</v>
@@ -2291,7 +2294,7 @@
       </c>
       <c r="H27" s="32"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
         <v>53</v>
@@ -2309,7 +2312,7 @@
       </c>
       <c r="H28" s="32"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1" t="s">
         <v>30</v>
@@ -2327,7 +2330,7 @@
       </c>
       <c r="H29" s="32"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
         <v>40</v>
@@ -2345,7 +2348,7 @@
       </c>
       <c r="H30" s="32"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
         <v>54</v>
@@ -2363,7 +2366,7 @@
       </c>
       <c r="H31" s="32"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="1" t="s">
         <v>34</v>
@@ -2381,7 +2384,7 @@
       </c>
       <c r="H32" s="32"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="1" t="s">
         <v>32</v>
@@ -2399,7 +2402,7 @@
       </c>
       <c r="H33" s="32"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1" t="s">
         <v>44</v>
@@ -2417,7 +2420,7 @@
       </c>
       <c r="H34" s="32"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="B35" s="1" t="s">
         <v>60</v>
@@ -2435,7 +2438,7 @@
       </c>
       <c r="H35" s="32"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1" t="s">
         <v>61</v>
@@ -2453,7 +2456,7 @@
       </c>
       <c r="H36" s="32"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" s="1" t="s">
         <v>45</v>
@@ -2471,7 +2474,7 @@
       </c>
       <c r="H37" s="32"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="46">
         <v>359</v>
       </c>
@@ -2491,7 +2494,7 @@
       </c>
       <c r="H38" s="32"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>788</v>
       </c>
@@ -2513,7 +2516,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1" t="s">
         <v>18</v>
@@ -2531,7 +2534,7 @@
       </c>
       <c r="H40" s="1"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>56</v>
       </c>
@@ -2551,7 +2554,7 @@
       </c>
       <c r="H41" s="1"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>359</v>
       </c>
@@ -2573,7 +2576,7 @@
       </c>
       <c r="H42" s="1"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>333</v>
       </c>
@@ -2595,7 +2598,7 @@
       </c>
       <c r="H43" s="32"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>339</v>
       </c>
@@ -2617,7 +2620,7 @@
       </c>
       <c r="H44" s="32"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>330</v>
       </c>
@@ -2639,7 +2642,7 @@
       </c>
       <c r="H45" s="1"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>58</v>
       </c>
@@ -2661,7 +2664,7 @@
       </c>
       <c r="H46" s="1"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>58</v>
       </c>
@@ -2685,7 +2688,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>58</v>
       </c>
@@ -2707,7 +2710,7 @@
       </c>
       <c r="H48" s="13"/>
     </row>
-    <row r="49" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="7">
         <v>333</v>
       </c>
@@ -2729,7 +2732,7 @@
       </c>
       <c r="H49" s="45"/>
     </row>
-    <row r="50" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="7">
         <v>339</v>
       </c>
@@ -2751,7 +2754,7 @@
       </c>
       <c r="H50" s="45"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="6">
         <v>339</v>
       </c>
@@ -2775,7 +2778,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="6">
         <v>333</v>
       </c>
@@ -2799,7 +2802,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" s="6">
         <v>330</v>
       </c>
@@ -2823,7 +2826,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="7">
         <v>330</v>
       </c>
@@ -2845,7 +2848,7 @@
       </c>
       <c r="H54" s="13"/>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="6">
         <v>359</v>
       </c>
@@ -2869,7 +2872,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="7">
         <v>359</v>
       </c>
@@ -2891,7 +2894,7 @@
       </c>
       <c r="H56" s="14"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>15</v>
       </c>
@@ -2913,7 +2916,7 @@
       </c>
       <c r="H57" s="1"/>
     </row>
-    <row r="58" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
         <v>15</v>
       </c>
@@ -2935,7 +2938,7 @@
       </c>
       <c r="H58" s="14"/>
     </row>
-    <row r="59" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="7" t="s">
         <v>15</v>
       </c>
@@ -2959,7 +2962,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="1"/>
       <c r="B60" s="1" t="s">
         <v>64</v>
@@ -2979,7 +2982,7 @@
       </c>
       <c r="H60" s="32"/>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>333</v>
       </c>
@@ -2999,7 +3002,7 @@
       </c>
       <c r="H61" s="32"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1" t="s">
         <v>65</v>
@@ -3019,7 +3022,7 @@
       </c>
       <c r="H62" s="32"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="1"/>
       <c r="B63" s="1" t="s">
         <v>66</v>
@@ -3039,7 +3042,7 @@
       </c>
       <c r="H63" s="32"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="1" t="s">
         <v>67</v>
@@ -3059,7 +3062,7 @@
       </c>
       <c r="H64" s="32"/>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
       <c r="B65" s="52" t="s">
         <v>68</v>
@@ -3079,7 +3082,7 @@
       </c>
       <c r="H65" s="32"/>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>771</v>
       </c>
@@ -3101,7 +3104,7 @@
       </c>
       <c r="H66" s="32"/>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" s="47"/>
       <c r="B67" s="47" t="s">
         <v>69</v>
@@ -3119,7 +3122,7 @@
       </c>
       <c r="H67" s="50"/>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" s="47"/>
       <c r="B68" s="47" t="s">
         <v>17</v>
@@ -3137,19 +3140,37 @@
       </c>
       <c r="H68" s="50"/>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A69" s="47"/>
-      <c r="B69" s="47"/>
-      <c r="C69" s="48"/>
-      <c r="D69" s="48"/>
-      <c r="E69" s="48">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" s="1"/>
+      <c r="B69" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F69" s="49">
+      <c r="F69" s="3">
+        <v>6</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H69" s="32"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" s="47"/>
+      <c r="B70" s="47"/>
+      <c r="C70" s="48"/>
+      <c r="D70" s="48"/>
+      <c r="E70" s="48">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="F70" s="49">
         <v>0</v>
       </c>
-      <c r="G69" s="47"/>
-      <c r="H69" s="50" t="s">
+      <c r="G70" s="47"/>
+      <c r="H70" s="50" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3171,17 +3192,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="10434906-596f-46a5-926f-3edb904f78ed" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5cf601e6-58d3-421d-924a-edb15cb4ffbe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010009CC3A6597A11045ABE4FD5F31EA711C" ma:contentTypeVersion="12" ma:contentTypeDescription="Opret et nyt dokument." ma:contentTypeScope="" ma:versionID="fa2c4518775dc96a615c1d2a158c0976">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5cf601e6-58d3-421d-924a-edb15cb4ffbe" xmlns:ns3="10434906-596f-46a5-926f-3edb904f78ed" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fad1a91493673d207d0fbfa855bc898b" ns2:_="" ns3:_="">
     <xsd:import namespace="5cf601e6-58d3-421d-924a-edb15cb4ffbe"/>
@@ -3382,6 +3392,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="10434906-596f-46a5-926f-3edb904f78ed" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5cf601e6-58d3-421d-924a-edb15cb4ffbe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DCB9C45-D152-4623-9B73-B6BC986385F0}">
   <ds:schemaRefs>
@@ -3391,19 +3412,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A179490C-0A0F-49E2-B446-73992CBF5C42}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b8a4b54d-5b65-4950-a991-6a7e15162dd0"/>
-    <ds:schemaRef ds:uri="974ded3a-0e14-4dac-a3a9-49794019817f"/>
-    <ds:schemaRef ds:uri="10434906-596f-46a5-926f-3edb904f78ed"/>
-    <ds:schemaRef ds:uri="5cf601e6-58d3-421d-924a-edb15cb4ffbe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C9C0377-D591-4653-82A6-BA2658B60FFD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3420,4 +3428,17 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A179490C-0A0F-49E2-B446-73992CBF5C42}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b8a4b54d-5b65-4950-a991-6a7e15162dd0"/>
+    <ds:schemaRef ds:uri="974ded3a-0e14-4dac-a3a9-49794019817f"/>
+    <ds:schemaRef ds:uri="10434906-596f-46a5-926f-3edb904f78ed"/>
+    <ds:schemaRef ds:uri="5cf601e6-58d3-421d-924a-edb15cb4ffbe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
New rule for flight type 321
</commit_message>
<xml_diff>
--- a/Indmødetal/Regler til Mie.xlsx
+++ b/Indmødetal/Regler til Mie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://serwizsystems.sharepoint.com/sites/DataogDigitalisering/Delte dokumenter/01_Lufthavn/Indmødetal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="389" documentId="8_{BD8435A5-424E-4FC5-929C-3243556E6BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87C19EE6-88D8-4F99-8344-432D29E54C38}"/>
+  <xr:revisionPtr revIDLastSave="394" documentId="8_{BD8435A5-424E-4FC5-929C-3243556E6BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9925A7F-492B-4735-ACB3-664D1A022C67}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{724EF2EA-7AA9-48FA-9EA3-9140F0F4E3A1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{724EF2EA-7AA9-48FA-9EA3-9140F0F4E3A1}"/>
   </bookViews>
   <sheets>
     <sheet name="wb" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="71">
   <si>
     <t>Tider WB Clean, search, guard</t>
   </si>
@@ -1049,10 +1049,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{62A5947B-93BF-4B94-A9B6-6F653D116F37}" name="Tabel1" displayName="Tabel1" ref="A1:H70" totalsRowShown="0" headerRowDxfId="9" tableBorderDxfId="8">
-  <autoFilter ref="A1:H70" xr:uid="{62A5947B-93BF-4B94-A9B6-6F653D116F37}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H37">
-    <sortCondition ref="B1:B37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{62A5947B-93BF-4B94-A9B6-6F653D116F37}" name="Tabel1" displayName="Tabel1" ref="A1:H71" totalsRowShown="0" headerRowDxfId="9" tableBorderDxfId="8">
+  <autoFilter ref="A1:H71" xr:uid="{62A5947B-93BF-4B94-A9B6-6F653D116F37}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H38">
+    <sortCondition ref="B1:B38"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{AF874BED-0EBC-4B8E-99D1-2C315245E3F5}" name="Flytype" dataDxfId="7"/>
@@ -1386,13 +1386,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4A27A0D-8896-47A0-95A9-30DD4012C6C3}">
   <dimension ref="B2:J19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="9" max="9" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" s="54" t="s">
         <v>0</v>
       </c>
@@ -1403,7 +1403,7 @@
       <c r="G2" s="54"/>
       <c r="H2" s="54"/>
     </row>
-    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
@@ -1432,7 +1432,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B4" s="25" t="s">
         <v>9</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B5" s="36" t="s">
         <v>9</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="37" t="s">
         <v>9</v>
       </c>
@@ -1507,7 +1507,7 @@
       <c r="I6" s="41"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" s="25" t="s">
         <v>13</v>
       </c>
@@ -1530,7 +1530,7 @@
       <c r="I7" s="11"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" s="36" t="s">
         <v>13</v>
       </c>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="37" t="s">
         <v>13</v>
       </c>
@@ -1578,7 +1578,7 @@
       <c r="I9" s="41"/>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B10" s="25" t="s">
         <v>15</v>
       </c>
@@ -1601,7 +1601,7 @@
       <c r="I10" s="11"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B11" s="36" t="s">
         <v>15</v>
       </c>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="J11" s="1"/>
     </row>
-    <row r="12" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="37" t="s">
         <v>15</v>
       </c>
@@ -1649,7 +1649,7 @@
       <c r="I12" s="42"/>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>16</v>
       </c>
@@ -1672,7 +1672,7 @@
       <c r="I13" s="15"/>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B14" s="21"/>
       <c r="C14" s="21" t="s">
         <v>18</v>
@@ -1693,7 +1693,7 @@
       <c r="I14" s="16"/>
       <c r="J14" s="1"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B15" s="21" t="s">
         <v>19</v>
       </c>
@@ -1716,7 +1716,7 @@
       <c r="I15" s="16"/>
       <c r="J15" s="1"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B16" s="21" t="s">
         <v>21</v>
       </c>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="2"/>
@@ -1752,7 +1752,7 @@
       <c r="I17" s="12"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C19" s="43" t="s">
         <v>62</v>
       </c>
@@ -1774,13 +1774,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D18F845-7CC0-4A12-B855-0E9D257F383F}">
-  <dimension ref="A1:H70"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H71"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="8" max="8" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>1</v>
       </c>
@@ -1806,7 +1806,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>35</v>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="H2" s="32"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>47</v>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="H3" s="32"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>39</v>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="H4" s="32"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>41</v>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="H5" s="32"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>59</v>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="H6" s="32"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>33</v>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="H7" s="32"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>58</v>
       </c>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="H8" s="32"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>57</v>
       </c>
@@ -1954,31 +1954,29 @@
       </c>
       <c r="H9" s="32"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
-        <v>339</v>
+        <v>321</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="2">
-        <v>1.0416666666666666E-2</v>
-      </c>
+      <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="2">
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="F10" s="3">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H10" s="32"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>31</v>
@@ -1998,9 +1996,9 @@
       </c>
       <c r="H11" s="32"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>31</v>
@@ -2020,71 +2018,75 @@
       </c>
       <c r="H12" s="32"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>330</v>
+      </c>
       <c r="B13" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="1"/>
+        <v>31</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1.0416666666666666E-2</v>
+      </c>
       <c r="D13" s="1"/>
       <c r="E13" s="2">
-        <v>1.0416666666666666E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="F13" s="3">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H13" s="32"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="2">
-        <v>1.0416666666666666E-2</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="2">
-        <v>3.125E-2</v>
+        <v>1.0416666666666666E-2</v>
       </c>
       <c r="F14" s="3">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H14" s="32"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="1"/>
+        <v>55</v>
+      </c>
+      <c r="C15" s="2">
+        <v>1.0416666666666666E-2</v>
+      </c>
       <c r="D15" s="1"/>
       <c r="E15" s="2">
-        <v>1.38888888888889E-2</v>
+        <v>3.125E-2</v>
       </c>
       <c r="F15" s="3">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H15" s="32"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="2">
-        <v>1.0416666666666666E-2</v>
+        <v>1.38888888888889E-2</v>
       </c>
       <c r="F16" s="3">
         <v>6</v>
@@ -2094,66 +2096,66 @@
       </c>
       <c r="H16" s="32"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>56</v>
-      </c>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="2">
-        <v>2.0833333333333332E-2</v>
+        <v>1.0416666666666666E-2</v>
       </c>
       <c r="F17" s="3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H17" s="32"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="B18" s="1" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="2">
-        <v>1.3888888888888888E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="F18" s="3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H18" s="32"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="2">
-        <v>6.9444444444444441E-3</v>
+        <v>1.3888888888888888E-2</v>
       </c>
       <c r="F19" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H19" s="32"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -2168,10 +2170,10 @@
       </c>
       <c r="H20" s="32"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -2186,10 +2188,10 @@
       </c>
       <c r="H21" s="32"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="1" t="s">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -2204,10 +2206,10 @@
       </c>
       <c r="H22" s="32"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -2215,71 +2217,71 @@
         <v>6.9444444444444441E-3</v>
       </c>
       <c r="F23" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H23" s="32"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="2">
-        <v>1.38888888888889E-2</v>
+        <v>6.9444444444444441E-3</v>
       </c>
       <c r="F24" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H24" s="32"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="2">
-        <v>1.0416666666666666E-2</v>
+        <v>1.38888888888889E-2</v>
       </c>
       <c r="F25" s="3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H25" s="32"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="2">
-        <v>6.9444444444444441E-3</v>
+        <v>1.0416666666666666E-2</v>
       </c>
       <c r="F26" s="3">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H26" s="32"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="1" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -2287,112 +2289,112 @@
         <v>6.9444444444444441E-3</v>
       </c>
       <c r="F27" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G27" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H27" s="32"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="2">
-        <v>1.3888888888888888E-2</v>
+        <v>6.9444444444444441E-3</v>
       </c>
       <c r="F28" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G28" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H28" s="32"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="1" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="2">
-        <v>6.9444444444444441E-3</v>
+        <v>1.3888888888888888E-2</v>
       </c>
       <c r="F29" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H29" s="32"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="1" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="2">
-        <v>1.3888888888888888E-2</v>
+        <v>6.9444444444444441E-3</v>
       </c>
       <c r="F30" s="3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G30" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H30" s="32"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="2">
-        <v>6.9444444444444441E-3</v>
+        <v>1.3888888888888888E-2</v>
       </c>
       <c r="F31" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H31" s="32"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="1" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" s="2">
-        <v>1.0416666666666666E-2</v>
+        <v>6.9444444444444441E-3</v>
       </c>
       <c r="F32" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H32" s="32"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
       <c r="E33" s="2">
-        <v>6.9444444444444441E-3</v>
+        <v>1.0416666666666666E-2</v>
       </c>
       <c r="F33" s="3">
         <v>6</v>
@@ -2402,15 +2404,15 @@
       </c>
       <c r="H33" s="32"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="1" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" s="2">
-        <v>1.38888888888889E-2</v>
+        <v>6.9444444444444441E-3</v>
       </c>
       <c r="F34" s="3">
         <v>6</v>
@@ -2420,15 +2422,15 @@
       </c>
       <c r="H34" s="32"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="2">
-        <v>1.0416666666666666E-2</v>
+        <v>1.38888888888889E-2</v>
       </c>
       <c r="F35" s="3">
         <v>6</v>
@@ -2438,15 +2440,15 @@
       </c>
       <c r="H35" s="32"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="2">
-        <v>2.0833333333333332E-2</v>
+        <v>1.0416666666666666E-2</v>
       </c>
       <c r="F36" s="3">
         <v>6</v>
@@ -2456,15 +2458,15 @@
       </c>
       <c r="H36" s="32"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="1" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="2">
-        <v>1.38888888888889E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="F37" s="3">
         <v>6</v>
@@ -2474,55 +2476,53 @@
       </c>
       <c r="H37" s="32"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="46">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="2">
+        <v>1.38888888888889E-2</v>
+      </c>
+      <c r="F38" s="3">
+        <v>6</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H38" s="32"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="46">
         <v>359</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B39" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C38" s="1"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="51">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="F38" s="33">
-        <v>12</v>
-      </c>
-      <c r="G38" s="34" t="s">
-        <v>10</v>
-      </c>
-      <c r="H38" s="32"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
-        <v>788</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="2"/>
-      <c r="E39" s="2">
-        <v>3.125E-2</v>
-      </c>
-      <c r="F39" s="3">
+      <c r="E39" s="51">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F39" s="33">
         <v>12</v>
       </c>
-      <c r="G39" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H39" s="35" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="1"/>
+      <c r="G39" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="H39" s="32"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>788</v>
+      </c>
       <c r="B40" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
+      <c r="D40" s="2"/>
       <c r="E40" s="2">
         <v>3.125E-2</v>
       </c>
@@ -2532,17 +2532,17 @@
       <c r="G40" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H40" s="1"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>56</v>
-      </c>
+      <c r="H40" s="35" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" s="1"/>
       <c r="B41" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C41" s="1"/>
-      <c r="D41" s="2"/>
+      <c r="D41" s="1"/>
       <c r="E41" s="2">
         <v>3.125E-2</v>
       </c>
@@ -2554,31 +2554,29 @@
       </c>
       <c r="H41" s="1"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="1"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2">
+        <v>3.125E-2</v>
+      </c>
+      <c r="F42" s="3">
+        <v>12</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H42" s="1"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
         <v>359</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C42" s="2">
-        <v>1.0416666666666666E-2</v>
-      </c>
-      <c r="D42" s="2"/>
-      <c r="E42" s="51">
-        <v>5.2083333333333336E-2</v>
-      </c>
-      <c r="F42" s="3">
-        <v>10</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H42" s="1"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="1">
-        <v>333</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>30</v>
@@ -2588,19 +2586,19 @@
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="51">
-        <v>4.1666666666666664E-2</v>
+        <v>5.2083333333333336E-2</v>
       </c>
       <c r="F43" s="3">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H43" s="32"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H43" s="1"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>30</v>
@@ -2620,9 +2618,9 @@
       </c>
       <c r="H44" s="32"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>30</v>
@@ -2640,11 +2638,11 @@
       <c r="G45" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H45" s="1"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>58</v>
+      <c r="H45" s="32"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46" s="1">
+        <v>330</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>30</v>
@@ -2657,62 +2655,62 @@
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="F46" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H46" s="1"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" s="6" t="s">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C47" s="1"/>
-      <c r="D47" s="2">
+      <c r="C47" s="2">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="D47" s="2"/>
+      <c r="E47" s="51">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F47" s="3">
+        <v>6</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H47" s="1"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C48" s="1"/>
+      <c r="D48" s="2">
         <v>6.25E-2</v>
       </c>
-      <c r="E47" s="2">
+      <c r="E48" s="2">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F47" s="3">
+      <c r="F48" s="3">
         <v>4</v>
       </c>
-      <c r="G47" s="1" t="s">
+      <c r="G48" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H47" s="12" t="s">
+      <c r="H48" s="12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="7" t="s">
+    <row r="49" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="7" t="s">
         <v>58</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C48" s="8"/>
-      <c r="D48" s="9">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="E48" s="9">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="F48" s="10">
-        <v>2</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H48" s="13"/>
-    </row>
-    <row r="49" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="7">
-        <v>333</v>
       </c>
       <c r="B49" s="8" t="s">
         <v>30</v>
@@ -2725,16 +2723,16 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="F49" s="10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G49" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H49" s="45"/>
-    </row>
-    <row r="50" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H49" s="13"/>
+    </row>
+    <row r="50" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="7">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="B50" s="8" t="s">
         <v>30</v>
@@ -2754,33 +2752,31 @@
       </c>
       <c r="H50" s="45"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="6">
+    <row r="51" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="7">
         <v>339</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C51" s="1"/>
-      <c r="D51" s="2">
-        <v>6.25E-2</v>
-      </c>
-      <c r="E51" s="2">
+      <c r="C51" s="8"/>
+      <c r="D51" s="9">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="E51" s="9">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F51" s="3">
-        <v>6</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H51" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F51" s="10">
+        <v>3</v>
+      </c>
+      <c r="G51" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H51" s="45"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="6">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>30</v>
@@ -2802,9 +2798,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="6">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>30</v>
@@ -2826,119 +2822,121 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="7">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A54" s="6">
         <v>330</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B54" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9">
+      <c r="C54" s="1"/>
+      <c r="D54" s="2">
+        <v>6.25E-2</v>
+      </c>
+      <c r="E54" s="2">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="F54" s="3">
+        <v>6</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H54" s="12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="7">
+        <v>330</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C55" s="8"/>
+      <c r="D55" s="9">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="E54" s="9">
+      <c r="E55" s="9">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F54" s="10">
+      <c r="F55" s="10">
         <v>3</v>
       </c>
-      <c r="G54" s="8" t="s">
+      <c r="G55" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H54" s="13"/>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" s="6">
+      <c r="H55" s="13"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A56" s="6">
         <v>359</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B56" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C55" s="1"/>
-      <c r="D55" s="2">
+      <c r="C56" s="1"/>
+      <c r="D56" s="2">
         <v>6.25E-2</v>
       </c>
-      <c r="E55" s="2">
+      <c r="E56" s="2">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F55" s="3">
+      <c r="F56" s="3">
         <v>6</v>
       </c>
-      <c r="G55" s="1" t="s">
+      <c r="G56" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H55" s="12" t="s">
+      <c r="H56" s="12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="7">
+    <row r="57" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="7">
         <v>359</v>
       </c>
-      <c r="B56" s="8" t="s">
+      <c r="B57" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C56" s="8"/>
-      <c r="D56" s="9">
+      <c r="C57" s="8"/>
+      <c r="D57" s="9">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="E56" s="9">
+      <c r="E57" s="9">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F56" s="8">
+      <c r="F57" s="8">
         <v>3</v>
       </c>
-      <c r="G56" s="8" t="s">
+      <c r="G57" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H56" s="14"/>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
+      <c r="H57" s="14"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B58" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C57" s="2">
+      <c r="C58" s="2">
         <v>1.0416666666666666E-2</v>
       </c>
-      <c r="D57" s="2"/>
-      <c r="E57" s="51">
+      <c r="D58" s="2"/>
+      <c r="E58" s="51">
         <v>5.2083333333333336E-2</v>
       </c>
-      <c r="F57" s="3">
-        <v>10</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H57" s="1"/>
-    </row>
-    <row r="58" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B58" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C58" s="8"/>
-      <c r="D58" s="9">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="E58" s="9">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="F58" s="8">
-        <v>3</v>
-      </c>
-      <c r="G58" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H58" s="14"/>
-    </row>
-    <row r="59" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F58" s="3">
+        <v>10</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H58" s="1"/>
+    </row>
+    <row r="59" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="7" t="s">
         <v>15</v>
       </c>
@@ -2946,70 +2944,72 @@
         <v>30</v>
       </c>
       <c r="C59" s="8"/>
-      <c r="D59" s="2">
+      <c r="D59" s="9">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="E59" s="9">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="F59" s="8">
+        <v>3</v>
+      </c>
+      <c r="G59" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H59" s="14"/>
+    </row>
+    <row r="60" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C60" s="8"/>
+      <c r="D60" s="2">
         <v>6.25E-2</v>
       </c>
-      <c r="E59" s="2">
+      <c r="E60" s="2">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F59" s="3">
+      <c r="F60" s="3">
         <v>6</v>
       </c>
-      <c r="G59" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H59" s="12" t="s">
+      <c r="H60" s="12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="1"/>
-      <c r="B60" s="1" t="s">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A61" s="1"/>
+      <c r="B61" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C60" s="2">
+      <c r="C61" s="2">
         <v>1.0416666666666666E-2</v>
       </c>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2">
-        <v>3.125E-2</v>
-      </c>
-      <c r="F60" s="3">
-        <v>10</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H60" s="32"/>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="1">
-        <v>333</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C61" s="1"/>
       <c r="D61" s="2"/>
       <c r="E61" s="2">
         <v>3.125E-2</v>
       </c>
       <c r="F61" s="3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H61" s="32"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A62" s="1"/>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
+        <v>333</v>
+      </c>
       <c r="B62" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C62" s="2">
-        <v>1.0416666666666666E-2</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C62" s="1"/>
       <c r="D62" s="2"/>
       <c r="E62" s="2">
         <v>3.125E-2</v>
@@ -3022,30 +3022,30 @@
       </c>
       <c r="H62" s="32"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C63" s="2">
-        <v>3.472222222222222E-3</v>
+        <v>1.0416666666666666E-2</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2">
-        <v>1.0416666666666666E-2</v>
+        <v>3.125E-2</v>
       </c>
       <c r="F63" s="3">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H63" s="32"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C64" s="2">
         <v>3.472222222222222E-3</v>
@@ -3062,115 +3062,135 @@
       </c>
       <c r="H64" s="32"/>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
-      <c r="B65" s="52" t="s">
+      <c r="B65" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C65" s="2">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="F65" s="3">
+        <v>4</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H65" s="32"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A66" s="1"/>
+      <c r="B66" s="52" t="s">
         <v>68</v>
       </c>
-      <c r="C65" s="51">
+      <c r="C66" s="51">
         <v>3.125E-2</v>
       </c>
-      <c r="D65" s="51"/>
-      <c r="E65" s="51">
+      <c r="D66" s="51"/>
+      <c r="E66" s="51">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="F65" s="53">
-        <v>10</v>
-      </c>
-      <c r="G65" s="52" t="s">
-        <v>10</v>
-      </c>
-      <c r="H65" s="32"/>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="1">
+      <c r="F66" s="53">
+        <v>10</v>
+      </c>
+      <c r="G66" s="52" t="s">
+        <v>10</v>
+      </c>
+      <c r="H66" s="32"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
         <v>771</v>
       </c>
-      <c r="B66" s="52" t="s">
+      <c r="B67" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="C66" s="51"/>
-      <c r="D66" s="51">
+      <c r="C67" s="51"/>
+      <c r="D67" s="51">
         <v>8.3333333333333329E-2</v>
       </c>
-      <c r="E66" s="51">
+      <c r="E67" s="51">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F66" s="53">
+      <c r="F67" s="53">
         <v>3</v>
       </c>
-      <c r="G66" s="52" t="s">
+      <c r="G67" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="H66" s="32"/>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A67" s="47"/>
-      <c r="B67" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="C67" s="48"/>
-      <c r="D67" s="48"/>
-      <c r="E67" s="48">
-        <v>6.9444444444444441E-3</v>
-      </c>
-      <c r="F67" s="49">
-        <v>4</v>
-      </c>
-      <c r="G67" s="47" t="s">
-        <v>10</v>
-      </c>
-      <c r="H67" s="50"/>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H67" s="32"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="47"/>
       <c r="B68" s="47" t="s">
-        <v>17</v>
+        <v>69</v>
       </c>
       <c r="C68" s="48"/>
       <c r="D68" s="48"/>
-      <c r="E68" s="2">
+      <c r="E68" s="48">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="F68" s="49">
+        <v>4</v>
+      </c>
+      <c r="G68" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="H68" s="50"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A69" s="47"/>
+      <c r="B69" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="C69" s="48"/>
+      <c r="D69" s="48"/>
+      <c r="E69" s="2">
         <v>3.125E-2</v>
       </c>
-      <c r="F68" s="3">
+      <c r="F69" s="3">
         <v>12</v>
       </c>
-      <c r="G68" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H68" s="50"/>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A69" s="1"/>
-      <c r="B69" s="1" t="s">
+      <c r="G69" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H69" s="50"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A70" s="1"/>
+      <c r="B70" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2">
+      <c r="C70" s="2"/>
+      <c r="D70" s="2"/>
+      <c r="E70" s="2">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F69" s="3">
+      <c r="F70" s="3">
         <v>6</v>
       </c>
-      <c r="G69" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H69" s="32"/>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A70" s="47"/>
-      <c r="B70" s="47"/>
-      <c r="C70" s="48"/>
-      <c r="D70" s="48"/>
-      <c r="E70" s="48">
+      <c r="G70" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H70" s="32"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A71" s="47"/>
+      <c r="B71" s="47"/>
+      <c r="C71" s="48"/>
+      <c r="D71" s="48"/>
+      <c r="E71" s="48">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="F70" s="49">
+      <c r="F71" s="49">
         <v>0</v>
       </c>
-      <c r="G70" s="47"/>
-      <c r="H70" s="50" t="s">
+      <c r="G71" s="47"/>
+      <c r="H71" s="50" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3192,6 +3212,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="10434906-596f-46a5-926f-3edb904f78ed" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5cf601e6-58d3-421d-924a-edb15cb4ffbe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010009CC3A6597A11045ABE4FD5F31EA711C" ma:contentTypeVersion="12" ma:contentTypeDescription="Opret et nyt dokument." ma:contentTypeScope="" ma:versionID="fa2c4518775dc96a615c1d2a158c0976">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5cf601e6-58d3-421d-924a-edb15cb4ffbe" xmlns:ns3="10434906-596f-46a5-926f-3edb904f78ed" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fad1a91493673d207d0fbfa855bc898b" ns2:_="" ns3:_="">
     <xsd:import namespace="5cf601e6-58d3-421d-924a-edb15cb4ffbe"/>
@@ -3392,17 +3423,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="10434906-596f-46a5-926f-3edb904f78ed" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5cf601e6-58d3-421d-924a-edb15cb4ffbe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5DCB9C45-D152-4623-9B73-B6BC986385F0}">
   <ds:schemaRefs>
@@ -3412,6 +3432,19 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A179490C-0A0F-49E2-B446-73992CBF5C42}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b8a4b54d-5b65-4950-a991-6a7e15162dd0"/>
+    <ds:schemaRef ds:uri="974ded3a-0e14-4dac-a3a9-49794019817f"/>
+    <ds:schemaRef ds:uri="10434906-596f-46a5-926f-3edb904f78ed"/>
+    <ds:schemaRef ds:uri="5cf601e6-58d3-421d-924a-edb15cb4ffbe"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C9C0377-D591-4653-82A6-BA2658B60FFD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3428,17 +3461,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A179490C-0A0F-49E2-B446-73992CBF5C42}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b8a4b54d-5b65-4950-a991-6a7e15162dd0"/>
-    <ds:schemaRef ds:uri="974ded3a-0e14-4dac-a3a9-49794019817f"/>
-    <ds:schemaRef ds:uri="10434906-596f-46a5-926f-3edb904f78ed"/>
-    <ds:schemaRef ds:uri="5cf601e6-58d3-421d-924a-edb15cb4ffbe"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>